<commit_message>
BLS: apply the MRI errata of August 2026 to the 4.0 file (#75)
The errata are authoritative until BLS 4.1, and fooddb serves the latest MRI data.
Only for a zip named BLS_4_0_*:

- Section 3: the oligosaccharides (OLSAC) were counted twice in the energy. For a
  food with OLSAC over 0, ENERC_KJ is ENERCJ - 8 x OLSAC and ENERC_KCAL is
  ENERCC - 2 x OLSAC. This is the 411 foods of appendix 7.4 (S151000: 413 kcal
  becomes 317.6). The OLSAC column must be in g.
- Section 6: no FAT, FASAT, ENERC_KJ or ENERC_KCAL for T104100 (Sardelle roh, 13.7 g
  fat, the MRI gives no new value) or the six entries of appendix 7.7 that are
  anchovy. The ten recipes with anchovy as a minor ingredient keep their values.

decisions.md says what is applied and why; tests use two more fixture rows.
</commit_message>
<xml_diff>
--- a/tests/fixtures/bls.xlsx
+++ b/tests/fixtures/bls.xlsx
@@ -191,6 +191,21 @@
           <t>NA Referenz</t>
         </is>
       </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>OLSAC Oligosaccharide, verfügbar [g/100g]</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>OLSAC Datenherkunft</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>OLSAC Referenz</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -373,26 +388,41 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>B121000</t>
+          <t>T104100</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Roggenvollkornbrot</t>
+          <t>Sardelle roh</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Wholemeal rye bread</t>
+          <t>Anchovy raw</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>812</t>
+          <t>849</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -407,7 +437,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>193</t>
+          <t>204</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -422,12 +452,12 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>46.4</t>
+          <t>75.3</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Analyse</t>
+          <t>Nährstoffdatenbank</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -437,12 +467,12 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>6.04</t>
+          <t>20.100000000000001</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Analyse</t>
+          <t>Nährstoffdatenbank</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -452,12 +482,12 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>1.81</t>
+          <t>13.7</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Analyse</t>
+          <t>Nährstoffdatenbank</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -467,7 +497,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>32.49</t>
+          <t>0</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -482,12 +512,12 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>9.6199999999999992</t>
+          <t>0</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Analyse</t>
+          <t>Logische Null</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
@@ -497,12 +527,12 @@
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>&lt;LOD</t>
+          <t>0</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>Analyse</t>
+          <t>Logische Null</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
@@ -512,7 +542,7 @@
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>4.58</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
@@ -527,7 +557,7 @@
       </c>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>0.187</t>
+          <t>4.3220000000000001</t>
         </is>
       </c>
       <c r="AF3" t="inlineStr">
@@ -542,15 +572,30 @@
       </c>
       <c r="AH3" t="inlineStr">
         <is>
-          <t>440.5</t>
+          <t>104</t>
         </is>
       </c>
       <c r="AI3" t="inlineStr">
         <is>
-          <t>Analyse</t>
+          <t>Nährstoffdatenbank</t>
         </is>
       </c>
       <c r="AJ3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AM3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -559,22 +604,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>R111000</t>
+          <t>B121000</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Speisesalz/Siedesalz/Tafelsalz</t>
+          <t>Roggenvollkornbrot</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Common salt/table salt</t>
+          <t>Wholemeal rye bread</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>812</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -589,7 +634,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>193</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -604,7 +649,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>0.1</t>
+          <t>46.4</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -619,12 +664,12 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6.04</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Logische Null</t>
+          <t>Analyse</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -634,12 +679,12 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1.81</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>Logische Null</t>
+          <t>Analyse</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -649,7 +694,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>32.49</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -664,12 +709,12 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>9.6199999999999992</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>Logische Null</t>
+          <t>Analyse</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
@@ -679,12 +724,12 @@
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>&lt;LOD</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>Logische Null</t>
+          <t>Analyse</t>
         </is>
       </c>
       <c r="AA4" t="inlineStr">
@@ -694,7 +739,7 @@
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4.58</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
@@ -709,7 +754,7 @@
       </c>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>0.187</t>
         </is>
       </c>
       <c r="AF4" t="inlineStr">
@@ -724,7 +769,7 @@
       </c>
       <c r="AH4" t="inlineStr">
         <is>
-          <t>38145</t>
+          <t>440.5</t>
         </is>
       </c>
       <c r="AI4" t="inlineStr">
@@ -733,6 +778,21 @@
         </is>
       </c>
       <c r="AJ4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AK4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AM4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -741,22 +801,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>P1A4000</t>
+          <t>R111000</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Leichtbier</t>
+          <t>Speisesalz/Siedesalz/Tafelsalz</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Light beer</t>
+          <t>Common salt/table salt</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>115</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -771,7 +831,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -786,12 +846,12 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>92.48</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Reskalierung</t>
+          <t>Analyse</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -801,12 +861,12 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>0.42199999999999999</t>
+          <t>0</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Reskalierung</t>
+          <t>Logische Null</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -821,7 +881,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>Reskalierung</t>
+          <t>Logische Null</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -831,7 +891,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>2.2000000000000002</t>
+          <t>0</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -851,7 +911,7 @@
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>Reskalierung</t>
+          <t>Logische Null</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
@@ -861,12 +921,12 @@
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>Labelangabe</t>
+          <t>Logische Null</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr">
@@ -876,12 +936,12 @@
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>0.1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>Reskalierung</t>
+          <t>Formelberechnung</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr">
@@ -906,15 +966,30 @@
       </c>
       <c r="AH5" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>38145</t>
         </is>
       </c>
       <c r="AI5" t="inlineStr">
         <is>
-          <t>Reskalierung</t>
+          <t>Analyse</t>
         </is>
       </c>
       <c r="AJ5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AK5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AL5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AM5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -923,22 +998,22 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Q180000</t>
+          <t>S151000</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Rapsöl/Rüböl</t>
+          <t>Glukosesirup maltosehaltig</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Rapeseed oil/canola oil</t>
+          <t>Glucose syrup containing maltose</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>3700</t>
+          <t>1733</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -953,7 +1028,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>413</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -968,12 +1043,12 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>20.5</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Spuren</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -998,12 +1073,12 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>0</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>Nährstoffdatenbank</t>
+          <t>Logische Null</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1013,7 +1088,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>79.5</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1028,29 +1103,29 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
           <t>Logische Null</t>
         </is>
       </c>
-      <c r="X6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="Z6" t="inlineStr">
-        <is>
-          <t>Logische Null</t>
-        </is>
-      </c>
       <c r="AA6" t="inlineStr">
         <is>
           <t>-</t>
@@ -1058,7 +1133,7 @@
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>31.8</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr">
@@ -1073,7 +1148,7 @@
       </c>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>7.2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AF6" t="inlineStr">
@@ -1088,15 +1163,30 @@
       </c>
       <c r="AH6" t="inlineStr">
         <is>
-          <t>1.65</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AI6" t="inlineStr">
         <is>
-          <t>Analyse</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AJ6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AK6" t="inlineStr">
+        <is>
+          <t>47.7</t>
+        </is>
+      </c>
+      <c r="AL6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AM6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1105,27 +1195,27 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Y999991</t>
+          <t>P1A4000</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Fixture</t>
+          <t>Leichtbier</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Fixture dish, traces and gaps</t>
+          <t>Light beer</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>115</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Analyse</t>
+          <t>Formelberechnung</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1135,12 +1225,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>27</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Analyse</t>
+          <t>Formelberechnung</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1150,12 +1240,12 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>92.48</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Fehlender Wert</t>
+          <t>Reskalierung</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1165,12 +1255,12 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0.42199999999999999</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Fehlender Wert</t>
+          <t>Reskalierung</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -1180,12 +1270,12 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>0</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>Analyse</t>
+          <t>Reskalierung</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1195,12 +1285,12 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>3.5</t>
+          <t>2.2000000000000002</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Analyse</t>
+          <t>Formelberechnung</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1210,12 +1300,12 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>Fehlender Wert</t>
+          <t>Reskalierung</t>
         </is>
       </c>
       <c r="X7" t="inlineStr">
@@ -1225,12 +1315,12 @@
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>Fehlender Wert</t>
+          <t>Labelangabe</t>
         </is>
       </c>
       <c r="AA7" t="inlineStr">
@@ -1240,12 +1330,12 @@
       </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>Fehlender Wert</t>
+          <t>Reskalierung</t>
         </is>
       </c>
       <c r="AD7" t="inlineStr">
@@ -1255,12 +1345,12 @@
       </c>
       <c r="AE7" t="inlineStr">
         <is>
-          <t>&lt;LOQ</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>Analyse</t>
+          <t>Formelberechnung</t>
         </is>
       </c>
       <c r="AG7" t="inlineStr">
@@ -1270,15 +1360,30 @@
       </c>
       <c r="AH7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="AI7" t="inlineStr">
         <is>
-          <t>Fehlender Wert</t>
+          <t>Reskalierung</t>
         </is>
       </c>
       <c r="AJ7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AK7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AL7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AM7" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1287,180 +1392,786 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>Q180000</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Rapsöl/Rüböl</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Rapeseed oil/canola oil</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>3700</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Formelberechnung</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>900</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Formelberechnung</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>TR</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Spuren</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Logische Null</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Nährstoffdatenbank</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Formelberechnung</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>Logische Null</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>Logische Null</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>Formelberechnung</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>7.2</t>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>Formelberechnung</t>
+        </is>
+      </c>
+      <c r="AG8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AH8" t="inlineStr">
+        <is>
+          <t>1.65</t>
+        </is>
+      </c>
+      <c r="AI8" t="inlineStr">
+        <is>
+          <t>Analyse</t>
+        </is>
+      </c>
+      <c r="AJ8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AK8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AL8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AM8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>W278400</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Schwedische Leberpastete mit Sardellen</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Swedish liver pate with anchovies</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>1101</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Formelberechnung</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>266</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Formelberechnung</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>60.7</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Rezeptberechnung</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>12.74</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Rezeptberechnung</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>23.2</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Rezeptberechnung</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Formelberechnung</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>Rezeptberechnung</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>Rezeptberechnung</t>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>Formelberechnung</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>Formelberechnung</t>
+        </is>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AH9" t="inlineStr">
+        <is>
+          <t>700</t>
+        </is>
+      </c>
+      <c r="AI9" t="inlineStr">
+        <is>
+          <t>Rezeptberechnung</t>
+        </is>
+      </c>
+      <c r="AJ9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AK9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AL9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AM9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Y999991</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Fixture</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Fixture dish, traces and gaps</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Analyse</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Analyse</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Fehlender Wert</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Fehlender Wert</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>TR</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Analyse</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>Analyse</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>Fehlender Wert</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>Fehlender Wert</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>Fehlender Wert</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>&lt;LOQ</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>Analyse</t>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AI10" t="inlineStr">
+        <is>
+          <t>Fehlender Wert</t>
+        </is>
+      </c>
+      <c r="AJ10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AK10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AL10" t="inlineStr">
+        <is>
+          <t>Fehlender Wert</t>
+        </is>
+      </c>
+      <c r="AM10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Y999992</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Leer</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Fixture dish without values</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>Fehlender Wert</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
         <is>
           <t>Fehlender Wert</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
         <is>
           <t>Fehlender Wert</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
         <is>
           <t>Fehlender Wert</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
         <is>
           <t>Fehlender Wert</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T8" t="inlineStr">
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
         <is>
           <t>Fehlender Wert</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W8" t="inlineStr">
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
         <is>
           <t>Fehlender Wert</t>
         </is>
       </c>
-      <c r="X8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Z8" t="inlineStr">
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
         <is>
           <t>Fehlender Wert</t>
         </is>
       </c>
-      <c r="AA8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AC8" t="inlineStr">
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
         <is>
           <t>Fehlender Wert</t>
         </is>
       </c>
-      <c r="AD8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AE8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AF8" t="inlineStr">
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF11" t="inlineStr">
         <is>
           <t>Fehlender Wert</t>
         </is>
       </c>
-      <c r="AG8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AH8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AI8" t="inlineStr">
+      <c r="AG11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AH11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AI11" t="inlineStr">
         <is>
           <t>Fehlender Wert</t>
         </is>
       </c>
-      <c r="AJ8" t="inlineStr">
+      <c r="AJ11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AK11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AL11" t="inlineStr">
+        <is>
+          <t>Fehlender Wert</t>
+        </is>
+      </c>
+      <c r="AM11" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>